<commit_message>
Phase 1: canonical categories + water failed-test recovery
New chemistry/scripts/categories.py encodes the approved rules: coffee→grains,
section-aware best-judgment, filter-water/شطة name groups. Integrated into
clean_chemistry.py, adding sample_category_canonical, category_flag,
sample_name_group to every parquet, plus water M1 recovery (invalid_test 2025 +
red-cell 2024 → failed_tests_derived).

Regenerated all 12 chemistry parquets + synced clean/chemistry/ (+ xlsx).
Suspect mislabels 107→12; coffee 181→grains; merges مياه فلتر 461 / شطة 132;
water failed-tests 41/46 (2024) + 54/64 (2025). Row parity preserved.
Supersedes clean/scripts/apply_category_canonical.py.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clean/chemistry/chem_honey_2025.xlsx
+++ b/clean/chemistry/chem_honey_2025.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'data'!$A$1:$BB$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'data'!$A$1:$BA$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB26"/>
+  <dimension ref="A1:BA26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -493,11 +493,10 @@
     <col width="14" customWidth="1" min="47" max="47"/>
     <col width="24" customWidth="1" min="48" max="48"/>
     <col width="40" customWidth="1" min="49" max="49"/>
-    <col width="12" customWidth="1" min="50" max="50"/>
-    <col width="12" customWidth="1" min="51" max="51"/>
-    <col width="27" customWidth="1" min="52" max="52"/>
-    <col width="24" customWidth="1" min="53" max="53"/>
-    <col width="10" customWidth="1" min="54" max="54"/>
+    <col width="17" customWidth="1" min="50" max="50"/>
+    <col width="27" customWidth="1" min="51" max="51"/>
+    <col width="15" customWidth="1" min="52" max="52"/>
+    <col width="25" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -748,27 +747,22 @@
       </c>
       <c r="AX1" s="1" t="inlineStr">
         <is>
-          <t>carb_qc</t>
+          <t>validity_status</t>
         </is>
       </c>
       <c r="AY1" s="1" t="inlineStr">
         <is>
-          <t>hmf_qc</t>
+          <t>sample_category_canonical</t>
         </is>
       </c>
       <c r="AZ1" s="1" t="inlineStr">
         <is>
-          <t>sample_category_canonical</t>
+          <t>category_flag</t>
         </is>
       </c>
       <c r="BA1" s="1" t="inlineStr">
         <is>
-          <t>municipality_canonical</t>
-        </is>
-      </c>
-      <c r="BB1" s="1" t="inlineStr">
-        <is>
-          <t>sector</t>
+          <t>sample_name_group</t>
         </is>
       </c>
     </row>
@@ -936,14 +930,19 @@
       <c r="AV2" t="n">
         <v>0</v>
       </c>
-      <c r="AZ2" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA2" t="inlineStr">
         <is>
-          <t>عينة خاصة</t>
+          <t>عسل عينة خاصة</t>
         </is>
       </c>
     </row>
@@ -1111,19 +1110,19 @@
       <c r="AV3" t="n">
         <v>0</v>
       </c>
-      <c r="AZ3" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA3" t="inlineStr">
         <is>
-          <t>الروضة</t>
-        </is>
-      </c>
-      <c r="BB3" t="inlineStr">
-        <is>
-          <t>East</t>
+          <t>عسل بشاور رقم 1</t>
         </is>
       </c>
     </row>
@@ -1296,19 +1295,19 @@
           <t>Sucrose</t>
         </is>
       </c>
-      <c r="AZ4" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA4" t="inlineStr">
         <is>
-          <t>الروضة</t>
-        </is>
-      </c>
-      <c r="BB4" t="inlineStr">
-        <is>
-          <t>East</t>
+          <t>عسل يمني</t>
         </is>
       </c>
     </row>
@@ -1471,14 +1470,19 @@
       <c r="AV5" t="n">
         <v>0</v>
       </c>
-      <c r="AZ5" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA5" t="inlineStr">
         <is>
-          <t>عينة خاصة</t>
+          <t>عسل عينة خاصة</t>
         </is>
       </c>
     </row>
@@ -1646,19 +1650,19 @@
           <t>HMF</t>
         </is>
       </c>
-      <c r="AZ6" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA6" t="inlineStr">
         <is>
-          <t>الروضة</t>
-        </is>
-      </c>
-      <c r="BB6" t="inlineStr">
-        <is>
-          <t>East</t>
+          <t>عسل زهور برية</t>
         </is>
       </c>
     </row>
@@ -1826,19 +1830,19 @@
           <t>Glucose + Fructose</t>
         </is>
       </c>
-      <c r="AZ7" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA7" t="inlineStr">
         <is>
-          <t>الروضة</t>
-        </is>
-      </c>
-      <c r="BB7" t="inlineStr">
-        <is>
-          <t>East</t>
+          <t>عسل طلح فاخر</t>
         </is>
       </c>
     </row>
@@ -1976,9 +1980,19 @@
       <c r="AV8" t="n">
         <v>0</v>
       </c>
-      <c r="AZ8" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>عينة خاصة عسل</t>
         </is>
       </c>
     </row>
@@ -2121,9 +2135,19 @@
           <t>Moisture|Acidity</t>
         </is>
       </c>
-      <c r="AZ9" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
+        </is>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>عينة خاصة دبس</t>
         </is>
       </c>
     </row>
@@ -2281,19 +2305,19 @@
       <c r="AV10" t="n">
         <v>0</v>
       </c>
-      <c r="AZ10" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA10" t="inlineStr">
         <is>
-          <t>العليا</t>
-        </is>
-      </c>
-      <c r="BB10" t="inlineStr">
-        <is>
-          <t>Central</t>
+          <t>عسل</t>
         </is>
       </c>
     </row>
@@ -2466,19 +2490,19 @@
           <t>Glucose + Fructose|HMF</t>
         </is>
       </c>
-      <c r="AZ11" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA11" t="inlineStr">
         <is>
-          <t>العليا</t>
-        </is>
-      </c>
-      <c r="BB11" t="inlineStr">
-        <is>
-          <t>Central</t>
+          <t>عسل</t>
         </is>
       </c>
     </row>
@@ -2651,19 +2675,19 @@
           <t>Glucose + Fructose</t>
         </is>
       </c>
-      <c r="AZ12" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA12" t="inlineStr">
         <is>
-          <t>الروضة</t>
-        </is>
-      </c>
-      <c r="BB12" t="inlineStr">
-        <is>
-          <t>East</t>
+          <t>عسل طبيعي</t>
         </is>
       </c>
     </row>
@@ -2828,19 +2852,19 @@
       <c r="AV13" t="n">
         <v>0</v>
       </c>
-      <c r="AZ13" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA13" t="inlineStr">
         <is>
-          <t>العليا</t>
-        </is>
-      </c>
-      <c r="BB13" t="inlineStr">
-        <is>
-          <t>Central</t>
+          <t>عسل م- ك</t>
         </is>
       </c>
     </row>
@@ -3003,19 +3027,19 @@
       <c r="AV14" t="n">
         <v>0</v>
       </c>
-      <c r="AZ14" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA14" t="inlineStr">
         <is>
-          <t>عرقة</t>
-        </is>
-      </c>
-      <c r="BB14" t="inlineStr">
-        <is>
-          <t>West</t>
+          <t>عسل سدر يمني م ك</t>
         </is>
       </c>
     </row>
@@ -3178,19 +3202,19 @@
       <c r="AV15" t="n">
         <v>0</v>
       </c>
-      <c r="AZ15" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA15" t="inlineStr">
         <is>
-          <t>عرقة</t>
-        </is>
-      </c>
-      <c r="BB15" t="inlineStr">
-        <is>
-          <t>West</t>
+          <t>عسل سدر م ك</t>
         </is>
       </c>
     </row>
@@ -3358,19 +3382,19 @@
           <t>Glucose + Fructose|Sucrose|HMF|Acidity</t>
         </is>
       </c>
-      <c r="AZ16" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA16" t="inlineStr">
         <is>
-          <t>الشمال</t>
-        </is>
-      </c>
-      <c r="BB16" t="inlineStr">
-        <is>
-          <t>North</t>
+          <t>عسل طبيعي</t>
         </is>
       </c>
     </row>
@@ -3533,19 +3557,19 @@
       <c r="AV17" t="n">
         <v>0</v>
       </c>
-      <c r="AZ17" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX17" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY17" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA17" t="inlineStr">
         <is>
-          <t>البطحاء</t>
-        </is>
-      </c>
-      <c r="BB17" t="inlineStr">
-        <is>
-          <t>Central</t>
+          <t>عسل سدر مستورد باكستاني</t>
         </is>
       </c>
     </row>
@@ -3718,19 +3742,19 @@
           <t>Glucose + Fructose|Sucrose</t>
         </is>
       </c>
-      <c r="AZ18" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX18" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA18" t="inlineStr">
         <is>
-          <t>البطحاء</t>
-        </is>
-      </c>
-      <c r="BB18" t="inlineStr">
-        <is>
-          <t>Central</t>
+          <t>عسل سدر حضرمي</t>
         </is>
       </c>
     </row>
@@ -3893,19 +3917,19 @@
       <c r="AV19" t="n">
         <v>0</v>
       </c>
-      <c r="AZ19" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX19" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA19" t="inlineStr">
         <is>
-          <t>البطحاء</t>
-        </is>
-      </c>
-      <c r="BB19" t="inlineStr">
-        <is>
-          <t>Central</t>
+          <t>عسل سدر بشاور</t>
         </is>
       </c>
     </row>
@@ -4068,19 +4092,19 @@
       <c r="AV20" t="n">
         <v>0</v>
       </c>
-      <c r="AZ20" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX20" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA20" t="inlineStr">
         <is>
-          <t>البطحاء</t>
-        </is>
-      </c>
-      <c r="BB20" t="inlineStr">
-        <is>
-          <t>Central</t>
+          <t>عسل زهور جبلي</t>
         </is>
       </c>
     </row>
@@ -4243,19 +4267,19 @@
       <c r="AV21" t="n">
         <v>0</v>
       </c>
-      <c r="AZ21" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY21" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA21" t="inlineStr">
         <is>
-          <t>البطحاء</t>
-        </is>
-      </c>
-      <c r="BB21" t="inlineStr">
-        <is>
-          <t>Central</t>
+          <t>عسل سدر اماراتي</t>
         </is>
       </c>
     </row>
@@ -4428,19 +4452,19 @@
           <t>HMF</t>
         </is>
       </c>
-      <c r="AZ22" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX22" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="AY22" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA22" t="inlineStr">
         <is>
-          <t>البطحاء</t>
-        </is>
-      </c>
-      <c r="BB22" t="inlineStr">
-        <is>
-          <t>Central</t>
+          <t>عسل سمره اماراتي</t>
         </is>
       </c>
     </row>
@@ -4613,19 +4637,19 @@
           <t>HMF</t>
         </is>
       </c>
-      <c r="AZ23" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX23" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="AY23" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA23" t="inlineStr">
         <is>
-          <t>البطحاء</t>
-        </is>
-      </c>
-      <c r="BB23" t="inlineStr">
-        <is>
-          <t>Central</t>
+          <t>عسل طلح محلي</t>
         </is>
       </c>
     </row>
@@ -4798,19 +4822,19 @@
           <t>HMF</t>
         </is>
       </c>
-      <c r="AZ24" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX24" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="AY24" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA24" t="inlineStr">
         <is>
-          <t>البطحاء</t>
-        </is>
-      </c>
-      <c r="BB24" t="inlineStr">
-        <is>
-          <t>Central</t>
+          <t>عسل حبة البركة مستورد</t>
         </is>
       </c>
     </row>
@@ -4973,19 +4997,19 @@
       <c r="AV25" t="n">
         <v>0</v>
       </c>
-      <c r="AZ25" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX25" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY25" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA25" t="inlineStr">
         <is>
-          <t>البطحاء</t>
-        </is>
-      </c>
-      <c r="BB25" t="inlineStr">
-        <is>
-          <t>Central</t>
+          <t>عسل شوكة يمني</t>
         </is>
       </c>
     </row>
@@ -5148,24 +5172,24 @@
       <c r="AV26" t="n">
         <v>0</v>
       </c>
-      <c r="AZ26" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل</t>
+      <c r="AX26" t="inlineStr">
+        <is>
+          <t>valid</t>
+        </is>
+      </c>
+      <c r="AY26" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل</t>
         </is>
       </c>
       <c r="BA26" t="inlineStr">
         <is>
-          <t>البطحاء</t>
-        </is>
-      </c>
-      <c r="BB26" t="inlineStr">
-        <is>
-          <t>Central</t>
+          <t>عسل برسيم مستورد من مصر</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BB26"/>
+  <autoFilter ref="A1:BA26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5176,7 +5200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -5202,7 +5226,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Columns: 54</t>
+          <t>Columns: 53</t>
         </is>
       </c>
     </row>
@@ -6093,82 +6117,68 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>carb_qc</t>
+          <t>validity_status</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="C55" t="n">
-        <v>25</v>
-      </c>
-      <c r="D55" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>valid | valid | valid</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>hmf_qc</t>
+          <t>sample_category_canonical</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="C56" t="n">
-        <v>25</v>
-      </c>
-      <c r="D56" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>الأطعمة الجاهزة للأكل | الأطعمة الجاهزة للأكل | الأطعمة الجاهزة للأكل</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>sample_category_canonical</t>
+          <t>category_flag</t>
         </is>
       </c>
       <c r="B57" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" t="n">
         <v>25</v>
       </c>
-      <c r="C57" t="n">
-        <v>0</v>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>الأطعمة الجاهزه للاكل | الأطعمة الجاهزه للاكل | الأطعمة الجاهزه للاكل</t>
-        </is>
-      </c>
+      <c r="D57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>municipality_canonical</t>
+          <t>sample_name_group</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>عينة خاصة | الروضة | الروضة</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>sector</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>21</v>
-      </c>
-      <c r="C59" t="n">
-        <v>4</v>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>East | East | East</t>
+          <t>عسل عينة خاصة | عسل بشاور رقم 1 | عسل يمني</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 1c: retire Ready-to-Eat category, honey→sweets
Per Muhannad: RTE→0 everywhere, nuts stay grains/legumes (GSO), honey→sweets,
other ex-RTE items reclassify by name. Removed RTE keyword + C_RTE from all
section valid-sets; routed عسل/دبس→sweets; added name rules for bread/flour/
onion/radish/mushroom/chips. RTE now 0, honey section 25→sweets, suspects 22→5.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clean/chemistry/chem_honey_2025.xlsx
+++ b/clean/chemistry/chem_honey_2025.xlsx
@@ -949,7 +949,7 @@
       </c>
       <c r="AY2" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA2" t="inlineStr">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="AY3" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA3" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="AY4" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA4" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="AY5" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA5" t="inlineStr">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="AY6" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA6" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="AY7" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA7" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="AY8" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA8" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="AY9" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA9" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="AY10" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA10" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="AY11" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA11" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="AY12" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA12" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="AY13" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA13" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="AY14" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA14" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="AY15" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA15" t="inlineStr">
@@ -3471,7 +3471,7 @@
       </c>
       <c r="AY16" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA16" t="inlineStr">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="AY17" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA17" t="inlineStr">
@@ -3841,7 +3841,7 @@
       </c>
       <c r="AY18" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA18" t="inlineStr">
@@ -4021,7 +4021,7 @@
       </c>
       <c r="AY19" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA19" t="inlineStr">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="AY20" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA20" t="inlineStr">
@@ -4381,7 +4381,7 @@
       </c>
       <c r="AY21" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA21" t="inlineStr">
@@ -4571,7 +4571,7 @@
       </c>
       <c r="AY22" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA22" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="AY23" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA23" t="inlineStr">
@@ -4951,7 +4951,7 @@
       </c>
       <c r="AY24" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA24" t="inlineStr">
@@ -5131,7 +5131,7 @@
       </c>
       <c r="AY25" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA25" t="inlineStr">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="AY26" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة</t>
         </is>
       </c>
       <c r="BA26" t="inlineStr">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>الأطعمة الجاهزة للأكل | الأطعمة الجاهزة للأكل | الأطعمة الجاهزة للأكل</t>
+          <t>الحلويات والشوكولاتة | الحلويات والشوكولاتة | الحلويات والشوكولاتة</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Chemistry: normalize municipality — merge private variants, clear out-of-place junk
Applied Muhannad's Sector_observed rulings: the three private-sample variants
(عينة خاصة / "( Private Sample) عينة خاصة" / ") عينة خاصة") merge to a single
«عينة خاصة» (168 rows); out-of-place values — product names / a stray number /
"NA"/"-" that leaked into the municipality field — are cleared and folded into
no_municipality (the former 21 "unmapped" rows). None location bucket unchanged
(3,433); 0 junk municipalities remain. Regenerated parquets + clean/chemistry
sync + xlsx + dashboard + validation workbook.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clean/chemistry/chem_honey_2025.xlsx
+++ b/clean/chemistry/chem_honey_2025.xlsx
@@ -839,7 +839,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>) عينة خاصة</t>
+          <t>عينة خاصة</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>) عينة خاصة</t>
+          <t>عينة خاصة</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -5647,7 +5647,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>) عينة خاصة | بلدية الروضة | بلدية الروضة</t>
+          <t>عينة خاصة | بلدية الروضة | بلدية الروضة</t>
         </is>
       </c>
     </row>

</xml_diff>